<commit_message>
Ajustados as configurações e limpeza dos dados
</commit_message>
<xml_diff>
--- a/data/extracao/ACORDO JUDICIAL.xlsx
+++ b/data/extracao/ACORDO JUDICIAL.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,12 +454,12 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>INDATA_INICIAL</t>
+          <t>MES</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>MES</t>
+          <t>MES_NOME</t>
         </is>
       </c>
     </row>
@@ -491,11 +487,13 @@
       <c r="G2" t="n">
         <v>99410.31</v>
       </c>
-      <c r="H2" s="1" t="n">
-        <v>45658</v>
-      </c>
-      <c r="I2" t="n">
+      <c r="H2" t="n">
         <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>JANEIRO</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -522,11 +520,13 @@
       <c r="G3" t="n">
         <v>38014.57</v>
       </c>
-      <c r="H3" s="1" t="n">
-        <v>45778</v>
-      </c>
-      <c r="I3" t="n">
+      <c r="H3" t="n">
         <v>5</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>MAIO</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -553,11 +553,13 @@
       <c r="G4" t="n">
         <v>3750</v>
       </c>
-      <c r="H4" s="1" t="n">
-        <v>45809</v>
-      </c>
-      <c r="I4" t="n">
+      <c r="H4" t="n">
         <v>6</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>JUNHO</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>